<commit_message>
feat: implement KTTV module with role-based access control, service layers, and integration testing suite
</commit_message>
<xml_diff>
--- a/docs/Bang_chuc_nang_theo_quyen_Cam_Pha.xlsx
+++ b/docs/Bang_chuc_nang_theo_quyen_Cam_Pha.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\SunSun\Documents\DuAN_20226\campha\server-campha\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{628D0238-618D-44E2-B4AB-9AC36E99CD05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D98E0248-4D2F-4024-A5BB-7D33B2A171B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Quy uoc quyen" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="428">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="449">
   <si>
     <t>PHỤ LỤC: BẢNG CHỨC NĂNG THEO QUYỀN NGƯỜI DÙNG - Hệ thống quản lý CSDL GIS đô thị hóa và hỗ trợ cảnh báo, giám sát ngập lụt, ngập úng thành phố Cẩm Phả trên nền tảng WebGIS và MobileGIS nhằm giảm nhẹ thiên tai</t>
   </si>
@@ -283,51 +283,7 @@
     <t>Thiết lập tham số mô hình thủy văn - thủy lực (Công việc 7.6)</t>
   </si>
   <si>
-    <t>(1) Khai báo phạm vi mô phỏng, lưới tính và bước thời gian
-(2) Nhập, chỉnh sửa bộ tham số mô hình thủy văn (mưa - dòng chảy) cho từng tiểu lưu vực
-(3) Nhập, chỉnh sửa bộ tham số mô hình thủy lực (lòng dẫn, công trình, điều kiện biên)
-(4) Tạo và quản lý các kịch bản mô phỏng (tần suất mưa thiết kế, tổ hợp mưa - triều, kịch bản đô thị hóa)
-(5) Hiệu chỉnh và kiểm định mô hình theo các trận lũ thực đo; tính các chỉ tiêu NSE, R2, PBIAS, RMSE
-(6) Lưu, sao chép, so sánh và khôi phục các bộ tham số theo phiên bản
-(7) Nhập/xuất bộ tham số dạng file (JSON, XML, CSV) để trao đổi với phần mềm mô hình chuyên dụng
-(8) Thiết lập ngưỡng cảnh báo ngập theo độ sâu, thời gian duy trì và diện tích ngập
-(9) Chạy thử mô hình và xem nhật ký lỗi, cảnh báo hội tụ</t>
-  </si>
-  <si>
-    <t>Giao diện chuyên gia cho phép cán bộ kỹ thuật khai báo toàn bộ thông số đầu vào của mô hình mưa - dòng chảy và mô hình diễn toán dòng chảy, thay vì phải sửa trực tiếp trong file cấu hình của phần mềm mô hình. Bộ tham số sau khi được hiệu chỉnh, kiểm định sẽ là đầu vào cho module Dự báo xu hướng phát triển các khu vực ngập lụt (mục 2.2, STT 10) và module Phân tích không gian (mục 2.2, STT 4). Chi tiết các tham số xem mục 4.1. Độ phức tạp: Phức tạp.</t>
-  </si>
-  <si>
-    <t>- Nhập, chỉnh sửa, chạy thử, hiệu chỉnh - kiểm định: TNMT, XD, QT
-- Tạo và ban hành kịch bản chính thức: chỉ TNMT
-- Xem bộ tham số và kết quả kiểm định: UB
-- Không cấp quyền cho: KH, ND</t>
-  </si>
-  <si>
     <t>10</t>
-  </si>
-  <si>
-    <t>Cấu hình tham số cho các lớp dữ liệu khí tượng thủy văn trực tuyến (Công việc 7.7)</t>
-  </si>
-  <si>
-    <t>(1) Khai báo nguồn dữ liệu khí tượng thủy văn trực tuyến (địa chỉ dịch vụ, khóa truy cập, định dạng trả về)
-(2) Kiểm tra kết nối và xem trước dữ liệu trả về từ nguồn
-(3) Cấu hình tham số không gian: phạm vi vùng nghiên cứu, ranh giới cắt dữ liệu, hệ tọa độ, phương pháp nội suy
-(4) Cấu hình tham số thời gian: chu kỳ cập nhật, múi giờ, thời hạn dự báo, thời gian lưu trữ chuỗi số liệu
-(5) Chọn biến khí tượng thủy văn cần lấy, khai báo đơn vị và hệ số quy đổi
-(6) Cấu hình hiển thị lớp dữ liệu: thang màu, ngưỡng phân cấp, độ trong suốt, thứ tự chồng lớp, tỷ lệ hiển thị
-(7) Quản lý danh mục trạm quan trắc trong và lân cận vùng nghiên cứu, thiết lập trọng số nội suy
-(8) Thiết lập quy tắc kiểm soát chất lượng số liệu và ngưỡng cảnh báo mưa, cấp báo động mực nước
-(9) Lập lịch thu thập tự động, khai báo nguồn dự phòng và xem nhật ký thu thập</t>
-  </si>
-  <si>
-    <t>Chức năng quản trị cho phép kết nối hệ thống với các dịch vụ khí tượng thủy văn trực tuyến (trạm quan trắc tự động, ảnh mưa vệ tinh, dữ liệu tái phân tích, dịch vụ dự báo thời tiết) và cấu hình để dữ liệu được cắt, nội suy, quy đổi đơn vị và hiển thị đúng cho phạm vi TP Cẩm Phả. Đây là nguồn cấp dữ liệu đầu vào thời gian thực cho mô hình ở Công việc 7.6, cho chức năng xem thời tiết trên Mobile GIS (mục 3, STT 1) và cho nghiệp vụ cảnh báo sớm. Chi tiết các tham số xem mục 4.2. Độ phức tạp: Phức tạp.</t>
-  </si>
-  <si>
-    <t>- Khai báo nguồn, cấu hình tham số không gian - thời gian - biến, lập lịch thu thập: TNMT, XD, QT
-- Cấu hình hiển thị lớp dữ liệu trên bản đồ (thang màu, chồng lớp): chỉ TNMT
-- Thiết lập ngưỡng cảnh báo và cấp báo động: TNMT, UB
-- Xem trạng thái kết nối và nhật ký thu thập: TNMT, UB, XD, QT
-- Không cấp quyền cho: KH, ND</t>
   </si>
   <si>
     <t>PHÂN HỆ WEB - NHÓM CHỨC NĂNG NGƯỜI DÙNG TRÊN WEBGIS (FRONT-END)</t>
@@ -579,9 +535,6 @@
     <t>CÔNG VIỆC 7.6 - THIẾT LẬP THAM SỐ MÔ HÌNH THỦY VĂN - THỦY LỰC</t>
   </si>
   <si>
-    <t>Chức năng này là màn hình khai báo dành cho cán bộ chuyên môn, phục vụ việc dựng và vận hành bộ đôi mô hình: mô hình thủy văn (chuyển mưa thành dòng chảy trên từng tiểu lưu vực) và mô hình thủy lực (diễn toán dòng chảy trong hệ thống kênh, mương, cống và tràn ra bề mặt để sinh bản đồ ngập). Toàn bộ tham số được lưu theo phiên bản và gắn với một kịch bản cụ thể, cho phép so sánh kết quả giữa các lần hiệu chỉnh. Các tham số cần nhập gồm:</t>
-  </si>
-  <si>
     <t>Nhóm tham số</t>
   </si>
   <si>
@@ -876,15 +829,9 @@
     <t>Ví dụ: mưa lớn trùng triều cường, mưa lớn khi triều kém</t>
   </si>
   <si>
-    <t>Tên kịch bản, người lập, ngày lập, ghi chú</t>
-  </si>
-  <si>
     <t>Văn bản</t>
   </si>
   <si>
-    <t>Phục vụ quản lý phiên bản</t>
-  </si>
-  <si>
     <t>5. Hiệu chỉnh và kiểm định</t>
   </si>
   <si>
@@ -939,12 +886,6 @@
     <t>Kết nối với module quản trị người dùng</t>
   </si>
   <si>
-    <t>CÔNG VIỆC 7.7 - CẤU HÌNH THAM SỐ CHO CÁC LỚP DỮ LIỆU KHÍ TƯỢNG THỦY VĂN TRỰC TUYẾN</t>
-  </si>
-  <si>
-    <t>Chức năng này không tạo ra dữ liệu mới mà làm nhiệm vụ kết nối và chuẩn hóa: lấy dữ liệu khí tượng thủy văn từ các dịch vụ trực tuyến bên ngoài, cắt về đúng phạm vi TP Cẩm Phả, nội suy về lưới tính của hệ thống, quy đổi đơn vị, kiểm soát chất lượng rồi công bố thành các lớp bản đồ động trên WebGIS và Mobile GIS. Mỗi nguồn dữ liệu được khai báo thành một cấu hình độc lập và có thể bật/tắt riêng. Các tham số cần nhập gồm:</t>
-  </si>
-  <si>
     <t>1. Khai báo nguồn dữ liệu</t>
   </si>
   <si>
@@ -1426,6 +1367,129 @@
   </si>
   <si>
     <t>- Hạ tầng máy chủ: PostgreSQL kèm phần mở rộng PostGIS; NodeJS với các thư viện Express, Socket.io, shapefile, TurfJS; chứng thư số HTTPS; hệ thống LDAP hoặc Active Directory của đơn vị chủ quản.</t>
+  </si>
+  <si>
+    <t>(1) Khai báo phạm vi mô phỏng, lưới tính và bước thời gian
+(2) Nhập, chỉnh sửa bộ tham số mô hình thủy văn (mưa - dòng chảy) cho từng tiểu lưu vực
+(3) Nhập, chỉnh sửa bộ tham số mô hình thủy lực (lòng dẫn, công trình, điều kiện biên)
+(4) Gắn bộ tham số đã phiên bản hóa vào kịch bản được chuẩn bị ở Công việc 7.7; không tạo lại danh mục kịch bản
+(5) Hiệu chỉnh và kiểm định mô hình theo các trận lũ thực đo; tính các chỉ tiêu NSE, R2, PBIAS, RMSE
+(6) Lưu, sao chép, so sánh và khôi phục các bộ tham số theo phiên bản
+(7) Nhập/xuất bộ tham số dạng file (JSON, XML, CSV) để trao đổi với phần mềm mô hình chuyên dụng
+(8) Thiết lập ngưỡng cảnh báo ngập theo độ sâu, thời gian duy trì và diện tích ngập
+(9) Chạy thử mô hình và xem nhật ký lỗi, cảnh báo hội tụ</t>
+  </si>
+  <si>
+    <t>Giao diện chuyên gia cho phép cán bộ kỹ thuật khai báo tham số mô hình mưa - dòng chảy và mô hình diễn toán dòng chảy. Danh mục kịch bản và quy tắc khớp được chuẩn bị trước ở Công việc 7.7; Công việc 7.6 gắn bộ tham số đã phiên bản hóa vào kịch bản đó, hiệu chỉnh, kiểm định và cung cấp đầu vào cho module dự báo ngập. Chi tiết các tham số xem mục 4.1. Độ phức tạp: Phức tạp.</t>
+  </si>
+  <si>
+    <t>- Nhập, chỉnh sửa, gắn bộ tham số, chạy thử, hiệu chỉnh - kiểm định: TNMT, XD, QT
+- Ban hành bộ tham số/kịch bản chính thức: chỉ TNMT
+- Xem bộ tham số và kết quả kiểm định: UB
+- Không cấp quyền cho: KH, ND</t>
+  </si>
+  <si>
+    <t>Tiếp nhận dữ liệu khí tượng thủy văn và chuẩn bị/khớp kịch bản (Công việc 7.7)</t>
+  </si>
+  <si>
+    <t>(1) Khai báo nguồn Weather API, khóa truy cập, định dạng trả về; kiểm tra kết nối và xem trước dữ liệu
+(2) Cấu hình tham số không gian, thời gian, biến, đơn vị, hệ số quy đổi và kiểm soát chất lượng
+(3) Quản lý danh mục trạm quan trắc, cấu hình hiển thị, ngưỡng cảnh báo và lịch thu thập
+(4) Chuẩn bị/nhập danh mục kịch bản do đơn vị nghiệp vụ cung cấp; cấu hình điều kiện khớp, mức ưu tiên, hiệu lực và phiên bản
+(5) Luồng tự động: lấy dữ liệu từ Weather API, chuẩn hóa rồi chọn kịch bản tương ứng
+(6) Luồng thủ công: nhập cùng bộ trường KTTV chuẩn, kiểm tra và chuẩn hóa rồi chọn kịch bản tương ứng
+(7) Dùng chung một bộ khớp cho hai luồng; dữ liệu đến không tự tạo kịch bản mới và không tự chạy mô hình
+(8) Trả trạng thái không khớp hoặc xung đột khi không có đúng một kịch bản phù hợp; lưu dữ liệu gốc, nguồn vào, người nhập và nhật ký khớp
+(9) Công bố lớp dữ liệu động lên WebGIS/Mobile GIS và gửi cảnh báo theo cấu hình</t>
+  </si>
+  <si>
+    <t>Chức năng quản trị tiếp nhận dữ liệu KTTV theo hai đường: tự động từ Weather API và nhập thủ công. Hai đường dùng cùng schema chuẩn hóa, kiểm soát chất lượng và bộ khớp để chọn một kịch bản đã được đơn vị nghiệp vụ chuẩn bị trong Sprint 10. Hệ thống không tự sinh kịch bản và chưa chạy engine mô hình ở bước này; bộ tham số được gắn ở Công việc 7.6 và mô hình chạy ở module dự báo ngập. Chi tiết tham số xem mục 4.2. Độ phức tạp: Phức tạp.</t>
+  </si>
+  <si>
+    <t>- Khai báo nguồn, cấu hình, quản lý trạm, lập lịch, nhập thủ công, chuẩn bị quy tắc và chạy khớp: TNMT, XD, QT
+- Ban hành/kích hoạt kịch bản chính thức: chỉ TNMT
+- Cấu hình hiển thị lớp dữ liệu: chỉ TNMT
+- Thiết lập ngưỡng cảnh báo và cấp báo động: TNMT, UB
+- Xem trạng thái, kết quả khớp và nhật ký: TNMT, UB, XD, QT
+- Không cấp quyền cho: KH, ND</t>
+  </si>
+  <si>
+    <t>Chức năng này là màn hình khai báo dành cho cán bộ chuyên môn, phục vụ dựng và vận hành mô hình thủy văn - thủy lực. Danh mục kịch bản và quy tắc khớp được đơn vị nghiệp vụ chuẩn bị trong Sprint 10 tại Công việc 7.7; màn hình này không tạo lại danh mục kịch bản mà gắn bộ tham số đã phiên bản hóa vào từng kịch bản để hiệu chỉnh, kiểm định và chạy mô hình. Các tham số cần nhập gồm:</t>
+  </si>
+  <si>
+    <t>Tên kịch bản tham chiếu, phiên bản kịch bản, bộ tham số gắn kèm, người lập, ngày lập, ghi chú</t>
+  </si>
+  <si>
+    <t>Kịch bản được chuẩn bị ở Công việc 7.7; chỉ TNMT ban hành/kích hoạt bản chính thức</t>
+  </si>
+  <si>
+    <t>CÔNG VIỆC 7.7 - TIẾP NHẬN DỮ LIỆU KHÍ TƯỢNG THỦY VĂN VÀ CHUẨN BỊ/KHỚP KỊCH BẢN</t>
+  </si>
+  <si>
+    <t>Chức năng này tiếp nhận dữ liệu khí tượng thủy văn theo hai luồng: tự động lấy từ Weather API hoặc nhập thủ công. Cả hai luồng dùng cùng bộ trường chuẩn, quy đổi đơn vị, kiểm soát chất lượng và bộ khớp để chọn một kịch bản do đơn vị nghiệp vụ chuẩn bị trong Sprint 10. Dữ liệu đến không tự tạo kịch bản mới; trường hợp không khớp hoặc khớp nhiều kịch bản phải dừng để xử lý. Mỗi nguồn và mỗi kịch bản có cấu hình độc lập, có phiên bản và có thể bật/tắt riêng. Các tham số cần nhập gồm:</t>
+  </si>
+  <si>
+    <t>8. Dữ liệu nhập thủ công</t>
+  </si>
+  <si>
+    <t>Bộ trường KTTV nhập thủ công</t>
+  </si>
+  <si>
+    <t>Cùng schema chuẩn hóa với Weather API</t>
+  </si>
+  <si>
+    <t>Gồm trạm/vị trí, thời điểm, biến, giá trị, đơn vị và ghi chú nguồn</t>
+  </si>
+  <si>
+    <t>Người nhập, thời điểm nhập và dữ liệu gốc</t>
+  </si>
+  <si>
+    <t>Nhật ký truy vết</t>
+  </si>
+  <si>
+    <t>Không cho sửa mất dấu vết nguồn vào</t>
+  </si>
+  <si>
+    <t>9. Kịch bản và quy tắc khớp</t>
+  </si>
+  <si>
+    <t>Tên, mã, phiên bản, hiệu lực và trạng thái kịch bản</t>
+  </si>
+  <si>
+    <t>Kịch bản do đơn vị nghiệp vụ chuẩn bị trong Sprint 10; chỉ TNMT ban hành/kích hoạt bản chính thức</t>
+  </si>
+  <si>
+    <t>Điều kiện khớp trên bộ biến KTTV chuẩn hóa</t>
+  </si>
+  <si>
+    <t>Dùng chung cho dữ liệu tự động và thủ công</t>
+  </si>
+  <si>
+    <t>Mức ưu tiên khi nhiều quy tắc cùng phù hợp</t>
+  </si>
+  <si>
+    <t>Số nguyên</t>
+  </si>
+  <si>
+    <t>Số nhỏ ưu tiên trước; cùng mức ưu tiên phải trả trạng thái xung đột</t>
+  </si>
+  <si>
+    <t>Kết quả khớp</t>
+  </si>
+  <si>
+    <t>matched / no_match / ambiguous</t>
+  </si>
+  <si>
+    <t>Không tự tạo kịch bản và không tự chạy mô hình</t>
+  </si>
+  <si>
+    <t>Bản chụp dữ liệu đầu vào và nguồn gốc</t>
+  </si>
+  <si>
+    <t>JSON/nhật ký</t>
+  </si>
+  <si>
+    <t>Lưu dữ liệu chuẩn hóa, automatic/manual, nguồn API hoặc người nhập</t>
   </si>
 </sst>
 </file>
@@ -1436,7 +1500,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -1847,28 +1911,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="78" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
     </row>
-    <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1879,7 +1943,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -1890,7 +1954,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1901,7 +1965,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
@@ -1912,7 +1976,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
@@ -1923,7 +1987,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>17</v>
       </c>
@@ -1934,7 +1998,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>20</v>
       </c>
@@ -1945,7 +2009,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>23</v>
       </c>
@@ -1968,7 +2032,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -1977,7 +2041,7 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>26</v>
       </c>
@@ -1986,7 +2050,7 @@
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
@@ -2003,7 +2067,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -2020,7 +2084,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>37</v>
       </c>
@@ -2037,7 +2101,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="90" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
@@ -2054,7 +2118,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
@@ -2071,7 +2135,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="105" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" ht="105" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>52</v>
       </c>
@@ -2088,7 +2152,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
@@ -2105,7 +2169,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
@@ -2122,7 +2186,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
@@ -2139,7 +2203,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" ht="240" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
@@ -2147,30 +2211,30 @@
         <v>71</v>
       </c>
       <c r="C12" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="300" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>75</v>
-      </c>
       <c r="B13" s="5" t="s">
-        <v>76</v>
+        <v>419</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>77</v>
+        <v>420</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>78</v>
+        <v>421</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>79</v>
+        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -2184,7 +2248,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E14"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -2193,16 +2257,16 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
@@ -2219,191 +2283,191 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="120" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="120" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>65</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C12" s="3" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="B14" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="D14" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2417,7 +2481,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
@@ -2426,16 +2490,16 @@
     <col min="5" max="5" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
       <c r="E1" s="8"/>
     </row>
-    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
@@ -2452,106 +2516,106 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="135" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>37</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>52</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>57</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2565,7 +2629,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D49"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
@@ -2573,560 +2637,560 @@
     <col min="4" max="4" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
     </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>145</v>
+        <v>423</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
     </row>
-    <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="3" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="3" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="3" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="3" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D9" s="3"/>
     </row>
-    <row r="10" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="3" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="3" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="3" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="3" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="D14" s="3"/>
     </row>
-    <row r="15" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="3" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="3" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="3" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5"/>
       <c r="B18" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="3" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D20" s="3"/>
     </row>
-    <row r="21" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="3" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="3" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5"/>
       <c r="B23" s="3" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D23" s="3"/>
     </row>
-    <row r="24" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="3" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="D24" s="3"/>
     </row>
-    <row r="25" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="3" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="3" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="D27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="3" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="D28" s="3"/>
     </row>
-    <row r="29" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5"/>
       <c r="B29" s="3" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="D29" s="3"/>
     </row>
-    <row r="30" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="D30" s="3"/>
     </row>
-    <row r="31" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="3" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5"/>
       <c r="B32" s="3" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="3" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
       <c r="B34" s="3" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="D34" s="3"/>
     </row>
-    <row r="35" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="3" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5"/>
       <c r="B37" s="3" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="3" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
       <c r="B39" s="3" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
       <c r="B40" s="3" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
       <c r="B41" s="3" t="s">
-        <v>244</v>
+        <v>424</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
       <c r="B43" s="3" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D43" s="3"/>
     </row>
-    <row r="44" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
       <c r="B44" s="3" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5"/>
       <c r="B45" s="3" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5"/>
       <c r="B47" s="3" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D47" s="3"/>
     </row>
-    <row r="48" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5"/>
       <c r="B48" s="3" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D48" s="3"/>
     </row>
-    <row r="49" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5"/>
       <c r="B49" s="3" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -3140,8 +3204,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D40"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D47"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="52" customWidth="1"/>
@@ -3149,462 +3213,550 @@
     <col min="4" max="4" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>265</v>
+        <v>426</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
     </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>266</v>
+        <v>427</v>
       </c>
       <c r="B2" s="8"/>
       <c r="C2" s="8"/>
       <c r="D2" s="8"/>
     </row>
-    <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5"/>
       <c r="B6" s="3" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="3" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D7" s="3"/>
     </row>
-    <row r="8" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5"/>
       <c r="B8" s="3" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="3" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5"/>
       <c r="B10" s="3" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="3" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="3" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
       <c r="D13" s="3"/>
     </row>
-    <row r="14" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="3" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="3" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="3" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>
       <c r="B17" s="3" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
       <c r="D17" s="3"/>
     </row>
-    <row r="18" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5"/>
       <c r="B19" s="3" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5"/>
       <c r="B20" s="3" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5"/>
       <c r="B21" s="3" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="D21" s="3"/>
     </row>
-    <row r="22" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5"/>
       <c r="B22" s="3" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="D22" s="3"/>
     </row>
-    <row r="23" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5"/>
       <c r="B24" s="3" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5"/>
       <c r="B25" s="3" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5"/>
       <c r="B26" s="3" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5"/>
       <c r="B27" s="3" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="D27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5"/>
       <c r="B28" s="3" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5"/>
       <c r="B30" s="3" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5"/>
       <c r="B31" s="3" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5"/>
       <c r="B33" s="3" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="D33" s="3"/>
     </row>
-    <row r="34" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5"/>
       <c r="B34" s="3" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="3" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5"/>
       <c r="B36" s="3" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
       <c r="D37" s="3"/>
     </row>
-    <row r="38" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
       <c r="B38" s="3" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="D38" s="3"/>
     </row>
-    <row r="39" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
       <c r="B39" s="3" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.2">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
       <c r="B40" s="3" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>352</v>
+        <v>340</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>353</v>
+        <v>341</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>428</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>430</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A42" s="5"/>
+      <c r="B42" s="5" t="s">
+        <v>432</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>433</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A44" s="5"/>
+      <c r="B44" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>322</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="5"/>
+      <c r="B46" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>444</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+      <c r="A47" s="5"/>
+      <c r="B47" s="5" t="s">
+        <v>446</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>447</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -3619,309 +3771,309 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C36"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="2" width="56" customWidth="1"/>
     <col min="3" max="3" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>354</v>
+        <v>342</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="8"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>347</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>351</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+    <row r="8" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>356</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>358</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>359</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>360</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>362</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>363</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>364</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>365</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>366</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>367</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>369</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>370</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>371</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>372</v>
+        <v>360</v>
       </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
     </row>
-    <row r="12" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>373</v>
+        <v>361</v>
       </c>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
     </row>
-    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>374</v>
+        <v>362</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
+        <v>367</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>370</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
+        <v>373</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>374</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+    <row r="20" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B20" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C20" s="3" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+    <row r="21" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>379</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
+    <row r="22" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
         <v>382</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B22" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="5" t="s">
+    <row r="23" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>385</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>386</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="5" t="s">
+    <row r="24" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
         <v>388</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="5" t="s">
+    <row r="25" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>391</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B25" s="3" t="s">
         <v>392</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C25" s="3" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="5" t="s">
+    <row r="26" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
         <v>394</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B26" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="C26" s="3" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="5" t="s">
+    <row r="27" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>397</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B27" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C27" s="3" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="5" t="s">
+    <row r="28" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
         <v>400</v>
       </c>
-      <c r="B24" s="3" t="s">
+      <c r="B28" s="3" t="s">
         <v>401</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="C28" s="3" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="5" t="s">
+    <row r="29" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>403</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B29" s="3" t="s">
         <v>404</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C29" s="3" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="5" t="s">
+    <row r="30" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="5" t="s">
         <v>406</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B30" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C30" s="3" t="s">
         <v>408</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
+    <row r="31" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>409</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B31" s="3" t="s">
         <v>410</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C31" s="3" t="s">
         <v>411</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="5" t="s">
-        <v>412</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="5" t="s">
-        <v>415</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="44.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="5" t="s">
-        <v>421</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>422</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>423</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>425</v>
+        <v>413</v>
       </c>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
     </row>
-    <row r="35" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>426</v>
+        <v>414</v>
       </c>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
     </row>
-    <row r="36" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" ht="33.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="11" t="s">
-        <v>427</v>
+        <v>415</v>
       </c>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>

</xml_diff>